<commit_message>
Adding the invoice to the exxcel file
</commit_message>
<xml_diff>
--- a/output/invoices.xlsx
+++ b/output/invoices.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,23 @@
         </is>
       </c>
       <c r="C3" t="inlineStr">
+        <is>
+          <t>B01101</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>صيدلية البهاء</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>906213079</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>B01101</t>
         </is>

</xml_diff>

<commit_message>
create server can receive HTTP request from Meta
</commit_message>
<xml_diff>
--- a/output/invoices.xlsx
+++ b/output/invoices.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,6 +481,60 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>B01101</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>صيدلية البهاء</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>906213079</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>B01101</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>30/09/2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>صيدلية البهاء</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>906213079</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>B01101</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>30.09.2020</t>
         </is>
       </c>
     </row>

</xml_diff>